<commit_message>
Reconcile all model sites and simplify data sharing
</commit_message>
<xml_diff>
--- a/data/processed/model_dataset.xlsx
+++ b/data/processed/model_dataset.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="R4bfbfb26574b49d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Data" sheetId="2" r:id="Rc2c6e7c9c80d4184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="Rc41d2089c5d64c99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Data" sheetId="2" r:id="R24c3e4cd73af4454"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -432,7 +432,7 @@
         <x:v>Current scope</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>49 observed sites: 44 ready for modelling and 5 requiring review.</x:v>
+        <x:v>49 observed sites: all 49 ready for modelling after source reconciliation.</x:v>
       </x:c>
       <x:c r="C5" s="21"/>
       <x:c r="D5" s="21"/>
@@ -472,7 +472,7 @@
         <x:v>Source basis</x:v>
       </x:c>
       <x:c r="B9" s="21" t="str">
-        <x:v>Client Ped_iRAP_merged.csv, raw survey workbooks and AusRAP road-segment data.</x:v>
+        <x:v>Client Ped_iRAP_merged.csv, archived raw survey workbooks, Road Network and AusRAP road-segment data.</x:v>
       </x:c>
       <x:c r="C9" s="21"/>
       <x:c r="D9" s="21"/>
@@ -482,7 +482,7 @@
         <x:v>Training rule</x:v>
       </x:c>
       <x:c r="B10" s="21" t="str">
-        <x:v>Filter qa_status = ready by default. Cross-validation splits are generated in code from site_id; do not edit this workbook into fixed train/test tabs.</x:v>
+        <x:v>Use all qa_status = ready rows. Generate cross-validation splits in code from site_id; report a sensitivity check excluding corrected-target sites 250341-04 and 260335-38.</x:v>
       </x:c>
       <x:c r="C10" s="21"/>
       <x:c r="D10" s="21"/>
@@ -512,7 +512,7 @@
         <x:v>Schema version</x:v>
       </x:c>
       <x:c r="B13" s="21" t="str">
-        <x:v>model_dataset_v1</x:v>
+        <x:v>model_dataset_v2</x:v>
       </x:c>
       <x:c r="C13" s="21"/>
       <x:c r="D13" s="21"/>
@@ -800,7 +800,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="D35" s="21" t="str">
-        <x:v>ready or review_required; training should use ready rows by default.</x:v>
+        <x:v>ready or review_required; all current rows are ready after source reconciliation.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
@@ -814,7 +814,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="D36" s="21" t="str">
-        <x:v>Reason a row requires reconciliation before training.</x:v>
+        <x:v>Reconciliation or audit note; a ready row may retain a documented correction.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2104,20 +2104,20 @@
       <x:c r="N22" s="30" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="O22" s="28" t="str">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="P22" s="28" t="str">
-        <x:v>25.5</x:v>
+      <x:c r="O22" s="28" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="P22" s="28" t="n">
+        <x:v>17.3333333333333</x:v>
       </x:c>
       <x:c r="Q22" s="27" t="str">
-        <x:v>Ped_iRAP_merged.csv</x:v>
+        <x:v>raw_survey_workbooks_three_day_reconstruction</x:v>
       </x:c>
       <x:c r="R22" s="27" t="str">
-        <x:v>review_required</x:v>
+        <x:v>ready</x:v>
       </x:c>
       <x:c r="S22" s="27" t="str">
-        <x:v>Schema-aware raw reconstruction does not reproduce the client-derived target. Confirm workbook layout and target derivation before model training.</x:v>
+        <x:v>Corrected from client compact values (125 cross, 25.5 along), which reproduce Thursday-Friday only; all three raw days and embedded hourly values give 87 cross and 17.3333 along.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -2515,10 +2515,10 @@
         <x:v>Ped_iRAP_merged.csv</x:v>
       </x:c>
       <x:c r="R29" s="27" t="str">
-        <x:v>review_required</x:v>
+        <x:v>ready</x:v>
       </x:c>
       <x:c r="S29" s="27" t="str">
-        <x:v>Client script uses M010; Road Network/AusRAP matching indicates H010. Standardised to H010 here; confirm the correction before model training.</x:v>
+        <x:v>Road code corrected from client M010 (Chidlow York Rd) to H010 (Coolgardie Esperance Hwy); Road Network contains SLK 366.85 on H010 and the raw targets reproduce.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2574,10 +2574,10 @@
         <x:v>Ped_iRAP_merged.csv</x:v>
       </x:c>
       <x:c r="R30" s="27" t="str">
-        <x:v>review_required</x:v>
+        <x:v>ready</x:v>
       </x:c>
       <x:c r="S30" s="27" t="str">
-        <x:v>Client script uses M010; Road Network/AusRAP matching indicates H010. Standardised to H010 here; confirm the correction before model training.</x:v>
+        <x:v>Road code corrected from client M010 (Chidlow York Rd) to H010 (Coolgardie Esperance Hwy); Road Network contains SLK 165.45 on H010 and the raw targets reproduce.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2911,17 +2911,17 @@
       <x:c r="O36" s="28" t="str">
         <x:v>4.33333333333333</x:v>
       </x:c>
-      <x:c r="P36" s="28" t="str">
-        <x:v>29.6666666666667</x:v>
+      <x:c r="P36" s="28" t="n">
+        <x:v>18.3333333333333</x:v>
       </x:c>
       <x:c r="Q36" s="27" t="str">
-        <x:v>Ped_iRAP_merged.csv</x:v>
+        <x:v>raw_survey_workbooks_schema_aware_reconstruction</x:v>
       </x:c>
       <x:c r="R36" s="27" t="str">
-        <x:v>review_required</x:v>
+        <x:v>ready</x:v>
       </x:c>
       <x:c r="S36" s="27" t="str">
-        <x:v>Special survey layout: schema-aware raw reconstruction does not reproduce the client-derived along-road target. Confirm the target before model training.</x:v>
+        <x:v>Corrected along target from 29.6667 to 18.3333; the special layout has one 15-minute along-road table, and its rolling result matches the embedded hourly values.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -3002,7 +3002,7 @@
         <x:v>North West Coastal Hwy</x:v>
       </x:c>
       <x:c r="H38" s="27" t="str">
-        <x:v>North West Coastal Hwy Norseman</x:v>
+        <x:v>North West Coastal Hwy Northampton</x:v>
       </x:c>
       <x:c r="I38" s="29" t="str">
         <x:v>-28.348677794</x:v>
@@ -3029,13 +3029,13 @@
         <x:v>66.33333333333333</x:v>
       </x:c>
       <x:c r="Q38" s="27" t="str">
-        <x:v>raw_survey_workbooks_reconstructed_client_rule</x:v>
+        <x:v>raw_survey_workbooks_three_day_reconstruction</x:v>
       </x:c>
       <x:c r="R38" s="27" t="str">
-        <x:v>review_required</x:v>
+        <x:v>ready</x:v>
       </x:c>
       <x:c r="S38" s="27" t="str">
-        <x:v>Location is absent from Ped_iRAP_merged.csv; targets reconstructed from three raw survey workbooks. Confirm before model training.</x:v>
+        <x:v>Absent from the client compact table; all three raw workbooks and embedded hourly values reproduce the targets. The workbook internal label resolves the filename's Norseman wording to NWCH Northampton.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -3725,7 +3725,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc012b1309bf43d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4821bab02f84876"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adopt Excel-only model data and add QA map
</commit_message>
<xml_diff>
--- a/data/processed/model_dataset.xlsx
+++ b/data/processed/model_dataset.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="Rc41d2089c5d64c99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Data" sheetId="2" r:id="R24c3e4cd73af4454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="Rd50ef221948a4386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Data" sheetId="2" r:id="R8ec9a46e60c44c9d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -422,7 +422,7 @@
         <x:v>Purpose</x:v>
       </x:c>
       <x:c r="B4" s="21" t="str">
-        <x:v>One row per surveyed site; this is the project’s model-development foundation table.</x:v>
+        <x:v>One row per surveyed site; this Excel workbook is the project’s authoritative model-development dataset.</x:v>
       </x:c>
       <x:c r="C4" s="21"/>
       <x:c r="D4" s="21"/>
@@ -660,7 +660,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="D25" s="21" t="str">
-        <x:v>Location wording preserved from the source survey filename.</x:v>
+        <x:v>Survey location label; an internal workbook label may correct a filename error.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -3725,7 +3725,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4821bab02f84876"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39d60579bc064b3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>